<commit_message>
dashboard kpi and other fixes
</commit_message>
<xml_diff>
--- a/public/templates/cosmetics/XLSX-Cosmetics Template.xlsx
+++ b/public/templates/cosmetics/XLSX-Cosmetics Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DIPAK\Desktop\Cosmetic Import Files\Sample files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152A4987-C457-4170-A494-0C43D2B99A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29B97CAA-CF67-497A-91C9-1041B5198EA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="XLSX-Cosmetics_Product_Upload" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="217">
   <si>
     <t>Product Category*</t>
   </si>
@@ -618,6 +618,120 @@
   </si>
   <si>
     <t>28% (for premium/luxury cosmetics) </t>
+  </si>
+  <si>
+    <t>Product Form</t>
+  </si>
+  <si>
+    <t>Liquid</t>
+  </si>
+  <si>
+    <t>Lotion</t>
+  </si>
+  <si>
+    <t>Serum</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>Spray</t>
+  </si>
+  <si>
+    <t>Mist</t>
+  </si>
+  <si>
+    <t>Foam</t>
+  </si>
+  <si>
+    <t>Cream</t>
+  </si>
+  <si>
+    <t>Gel</t>
+  </si>
+  <si>
+    <t>Paste</t>
+  </si>
+  <si>
+    <t>Balm</t>
+  </si>
+  <si>
+    <t>Wax</t>
+  </si>
+  <si>
+    <t>Powder</t>
+  </si>
+  <si>
+    <t>Solid</t>
+  </si>
+  <si>
+    <t>Stick</t>
+  </si>
+  <si>
+    <t>Roll-On</t>
+  </si>
+  <si>
+    <t>Tablet</t>
+  </si>
+  <si>
+    <t>Capsule</t>
+  </si>
+  <si>
+    <t>Sachet</t>
+  </si>
+  <si>
+    <t>Wipes</t>
+  </si>
+  <si>
+    <t>Patch</t>
+  </si>
+  <si>
+    <t>Soap Bar</t>
+  </si>
+  <si>
+    <t>Kit</t>
+  </si>
+  <si>
+    <t>Set</t>
+  </si>
+  <si>
+    <t>Millilitre (ml)</t>
+  </si>
+  <si>
+    <t>Litre (L)</t>
+  </si>
+  <si>
+    <t>Milligram (mg)</t>
+  </si>
+  <si>
+    <t>Gram (g)</t>
+  </si>
+  <si>
+    <t>Kilogram (kg)</t>
+  </si>
+  <si>
+    <t>Tablet(s)</t>
+  </si>
+  <si>
+    <t>Capsule(s)</t>
+  </si>
+  <si>
+    <t>Sachet(s)</t>
+  </si>
+  <si>
+    <t>Sheet(s)</t>
+  </si>
+  <si>
+    <t>Patch(es)</t>
+  </si>
+  <si>
+    <t>Unit(s)</t>
+  </si>
+  <si>
+    <t>Net Quantity Unit*</t>
+  </si>
+  <si>
+    <t>Product Form*</t>
   </si>
 </sst>
 </file>
@@ -703,7 +817,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -717,15 +831,16 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -853,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BJ2"/>
+  <dimension ref="A1:BL2"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
@@ -889,284 +1004,297 @@
     <col min="31" max="31" width="17.33203125" customWidth="1"/>
     <col min="32" max="32" width="11" customWidth="1"/>
     <col min="33" max="33" width="11.44140625" customWidth="1"/>
-    <col min="34" max="34" width="17.109375" customWidth="1"/>
-    <col min="35" max="35" width="24.5546875" customWidth="1"/>
-    <col min="36" max="36" width="18.6640625" customWidth="1"/>
-    <col min="37" max="37" width="17.5546875" customWidth="1"/>
-    <col min="38" max="38" width="17.88671875" customWidth="1"/>
-    <col min="39" max="39" width="16.88671875" customWidth="1"/>
-    <col min="40" max="40" width="17.109375" customWidth="1"/>
-    <col min="41" max="41" width="25.5546875" customWidth="1"/>
-    <col min="42" max="42" width="24.5546875" customWidth="1"/>
-    <col min="43" max="43" width="18.6640625" customWidth="1"/>
-    <col min="44" max="44" width="17.5546875" customWidth="1"/>
-    <col min="45" max="45" width="17.88671875" customWidth="1"/>
-    <col min="46" max="46" width="16.88671875" customWidth="1"/>
-    <col min="47" max="47" width="17.109375" customWidth="1"/>
-    <col min="48" max="48" width="25.5546875" customWidth="1"/>
-    <col min="49" max="49" width="24.5546875" customWidth="1"/>
-    <col min="50" max="50" width="18.6640625" customWidth="1"/>
-    <col min="51" max="51" width="17.5546875" customWidth="1"/>
-    <col min="52" max="52" width="17.88671875" customWidth="1"/>
-    <col min="53" max="53" width="16.88671875" customWidth="1"/>
-    <col min="54" max="54" width="17.109375" customWidth="1"/>
-    <col min="55" max="55" width="25.5546875" customWidth="1"/>
-    <col min="56" max="56" width="24.5546875" customWidth="1"/>
-    <col min="57" max="57" width="18.6640625" customWidth="1"/>
-    <col min="58" max="58" width="17.5546875" customWidth="1"/>
-    <col min="59" max="59" width="17.88671875" customWidth="1"/>
-    <col min="60" max="60" width="16.88671875" customWidth="1"/>
-    <col min="61" max="61" width="17.109375" customWidth="1"/>
-    <col min="62" max="62" width="18.109375" customWidth="1"/>
+    <col min="34" max="34" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="17.109375" customWidth="1"/>
+    <col min="37" max="37" width="24.5546875" customWidth="1"/>
+    <col min="38" max="38" width="18.6640625" customWidth="1"/>
+    <col min="39" max="39" width="17.5546875" customWidth="1"/>
+    <col min="40" max="40" width="17.88671875" customWidth="1"/>
+    <col min="41" max="41" width="16.88671875" customWidth="1"/>
+    <col min="42" max="42" width="17.109375" customWidth="1"/>
+    <col min="43" max="43" width="25.5546875" customWidth="1"/>
+    <col min="44" max="44" width="24.5546875" customWidth="1"/>
+    <col min="45" max="45" width="18.6640625" customWidth="1"/>
+    <col min="46" max="46" width="17.5546875" customWidth="1"/>
+    <col min="47" max="47" width="17.88671875" customWidth="1"/>
+    <col min="48" max="48" width="16.88671875" customWidth="1"/>
+    <col min="49" max="49" width="17.109375" customWidth="1"/>
+    <col min="50" max="50" width="25.5546875" customWidth="1"/>
+    <col min="51" max="51" width="24.5546875" customWidth="1"/>
+    <col min="52" max="52" width="18.6640625" customWidth="1"/>
+    <col min="53" max="53" width="17.5546875" customWidth="1"/>
+    <col min="54" max="54" width="17.88671875" customWidth="1"/>
+    <col min="55" max="55" width="16.88671875" customWidth="1"/>
+    <col min="56" max="56" width="17.109375" customWidth="1"/>
+    <col min="57" max="57" width="25.5546875" customWidth="1"/>
+    <col min="58" max="58" width="24.5546875" customWidth="1"/>
+    <col min="59" max="59" width="18.6640625" customWidth="1"/>
+    <col min="60" max="60" width="17.5546875" customWidth="1"/>
+    <col min="61" max="61" width="17.88671875" customWidth="1"/>
+    <col min="62" max="62" width="16.88671875" customWidth="1"/>
+    <col min="63" max="63" width="17.109375" customWidth="1"/>
+    <col min="64" max="64" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:64" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="U1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="V1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="W1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="X1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Y1" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="9" t="s">
+      <c r="Z1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="9" t="s">
+      <c r="AA1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AB1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AC1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AD1" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AE1" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AF1" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AG1" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" t="s">
+      <c r="AH1" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="AI1" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="AJ1" t="s">
         <v>33</v>
       </c>
-      <c r="AO1" t="s">
+      <c r="AQ1" t="s">
         <v>34</v>
       </c>
-      <c r="AV1" t="s">
+      <c r="AX1" t="s">
         <v>34</v>
       </c>
-      <c r="BC1" t="s">
+      <c r="BE1" t="s">
         <v>34</v>
       </c>
-      <c r="BJ1" t="s">
+      <c r="BL1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:62" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="9"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="9"/>
-      <c r="O2" s="9"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
-      <c r="S2" s="9"/>
-      <c r="T2" s="9"/>
-      <c r="U2" s="9"/>
-      <c r="V2" s="9"/>
-      <c r="W2" s="9"/>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="9"/>
-      <c r="Z2" s="9"/>
-      <c r="AA2" s="9"/>
-      <c r="AB2" s="9"/>
-      <c r="AC2" s="9"/>
-      <c r="AD2" s="9"/>
-      <c r="AE2" s="9"/>
-      <c r="AF2" s="9"/>
-      <c r="AG2" s="9"/>
-      <c r="AH2" t="s">
+    <row r="2" spans="1:64" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11"/>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11"/>
+      <c r="R2" s="11"/>
+      <c r="S2" s="11"/>
+      <c r="T2" s="11"/>
+      <c r="U2" s="11"/>
+      <c r="V2" s="11"/>
+      <c r="W2" s="11"/>
+      <c r="X2" s="11"/>
+      <c r="Y2" s="11"/>
+      <c r="Z2" s="11"/>
+      <c r="AA2" s="11"/>
+      <c r="AB2" s="11"/>
+      <c r="AC2" s="11"/>
+      <c r="AD2" s="11"/>
+      <c r="AE2" s="11"/>
+      <c r="AF2" s="11"/>
+      <c r="AG2" s="11"/>
+      <c r="AH2" s="11"/>
+      <c r="AI2" s="11"/>
+      <c r="AJ2" t="s">
         <v>36</v>
       </c>
-      <c r="AI2" t="s">
+      <c r="AK2" t="s">
         <v>37</v>
       </c>
-      <c r="AJ2" t="s">
+      <c r="AL2" t="s">
         <v>38</v>
       </c>
-      <c r="AK2" t="s">
+      <c r="AM2" t="s">
         <v>39</v>
       </c>
-      <c r="AL2" t="s">
+      <c r="AN2" t="s">
         <v>40</v>
       </c>
-      <c r="AM2" t="s">
+      <c r="AO2" t="s">
         <v>41</v>
       </c>
-      <c r="AN2" t="s">
+      <c r="AP2" t="s">
         <v>42</v>
       </c>
-      <c r="AO2" t="s">
+      <c r="AQ2" t="s">
         <v>36</v>
       </c>
-      <c r="AP2" t="s">
+      <c r="AR2" t="s">
         <v>37</v>
       </c>
-      <c r="AQ2" t="s">
+      <c r="AS2" t="s">
         <v>38</v>
       </c>
-      <c r="AR2" t="s">
+      <c r="AT2" t="s">
         <v>39</v>
       </c>
-      <c r="AS2" t="s">
+      <c r="AU2" t="s">
         <v>40</v>
       </c>
-      <c r="AT2" t="s">
+      <c r="AV2" t="s">
         <v>41</v>
       </c>
-      <c r="AU2" t="s">
+      <c r="AW2" t="s">
         <v>42</v>
       </c>
-      <c r="AV2" t="s">
+      <c r="AX2" t="s">
         <v>36</v>
       </c>
-      <c r="AW2" t="s">
+      <c r="AY2" t="s">
         <v>37</v>
       </c>
-      <c r="AX2" t="s">
+      <c r="AZ2" t="s">
         <v>38</v>
       </c>
-      <c r="AY2" t="s">
+      <c r="BA2" t="s">
         <v>39</v>
       </c>
-      <c r="AZ2" t="s">
+      <c r="BB2" t="s">
         <v>40</v>
       </c>
-      <c r="BA2" t="s">
+      <c r="BC2" t="s">
         <v>41</v>
       </c>
-      <c r="BB2" t="s">
+      <c r="BD2" t="s">
         <v>42</v>
       </c>
-      <c r="BC2" t="s">
+      <c r="BE2" t="s">
         <v>36</v>
       </c>
-      <c r="BD2" t="s">
+      <c r="BF2" t="s">
         <v>37</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="BG2" t="s">
         <v>38</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BH2" t="s">
         <v>39</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BI2" t="s">
         <v>40</v>
       </c>
-      <c r="BH2" t="s">
+      <c r="BJ2" t="s">
         <v>41</v>
       </c>
-      <c r="BI2" t="s">
+      <c r="BK2" t="s">
         <v>42</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="AD1:AD2"/>
-    <mergeCell ref="AE1:AE2"/>
-    <mergeCell ref="AF1:AF2"/>
-    <mergeCell ref="AG1:AG2"/>
-    <mergeCell ref="X1:X2"/>
-    <mergeCell ref="Y1:Y2"/>
-    <mergeCell ref="Z1:Z2"/>
-    <mergeCell ref="AA1:AA2"/>
-    <mergeCell ref="AB1:AB2"/>
-    <mergeCell ref="AC1:AC2"/>
+  <mergeCells count="35">
+    <mergeCell ref="AH1:AH2"/>
+    <mergeCell ref="AI1:AI2"/>
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="W1:W2"/>
     <mergeCell ref="L1:L2"/>
     <mergeCell ref="M1:M2"/>
@@ -1179,17 +1307,16 @@
     <mergeCell ref="T1:T2"/>
     <mergeCell ref="U1:U2"/>
     <mergeCell ref="V1:V2"/>
-    <mergeCell ref="K1:K2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
+    <mergeCell ref="AD1:AD2"/>
+    <mergeCell ref="AE1:AE2"/>
+    <mergeCell ref="AF1:AF2"/>
+    <mergeCell ref="AG1:AG2"/>
+    <mergeCell ref="X1:X2"/>
+    <mergeCell ref="Y1:Y2"/>
+    <mergeCell ref="Z1:Z2"/>
+    <mergeCell ref="AA1:AA2"/>
+    <mergeCell ref="AB1:AB2"/>
+    <mergeCell ref="AC1:AC2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -1202,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1A2E768-424D-4C07-879C-980AF9B93D86}">
-  <dimension ref="A1:T62"/>
+  <dimension ref="A1:X62"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -1216,9 +1343,11 @@
     <col min="16" max="16" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="37.44140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.21875" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1250,12 +1379,18 @@
       <c r="T1" s="3" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V1" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="X1" s="12" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="9" t="s">
         <v>46</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -1285,12 +1420,18 @@
       <c r="T2" s="4" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V2" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="11"/>
+      <c r="C3" s="9"/>
       <c r="D3" s="2" t="s">
         <v>73</v>
       </c>
@@ -1318,12 +1459,18 @@
       <c r="T3" s="4" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="4" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V3" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C4" s="11"/>
+      <c r="C4" s="9"/>
       <c r="D4" s="2" t="s">
         <v>72</v>
       </c>
@@ -1351,12 +1498,18 @@
       <c r="T4" s="4" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="5" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V4" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="11"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="2" t="s">
         <v>76</v>
       </c>
@@ -1381,12 +1534,18 @@
       <c r="T5" s="4" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="6" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V5" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="X5" s="2" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="11"/>
+      <c r="C6" s="9"/>
       <c r="D6" s="2" t="s">
         <v>75</v>
       </c>
@@ -1411,12 +1570,18 @@
       <c r="T6" s="4" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="7" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V6" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="X6" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="11"/>
+      <c r="C7" s="9"/>
       <c r="D7" s="2" t="s">
         <v>78</v>
       </c>
@@ -1438,12 +1603,18 @@
       <c r="R7" s="8" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V7" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="X7" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C8" s="11"/>
+      <c r="C8" s="9"/>
       <c r="D8" s="2" t="s">
         <v>77</v>
       </c>
@@ -1456,12 +1627,18 @@
       <c r="R8" s="8" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="9" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V8" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="9" t="s">
         <v>49</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1476,12 +1653,18 @@
       <c r="R9" s="8" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="10" spans="1:20" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="V9" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C10" s="11"/>
+      <c r="C10" s="9"/>
       <c r="D10" s="2" t="s">
         <v>87</v>
       </c>
@@ -1491,18 +1674,30 @@
       <c r="R10" s="8" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C11" s="11"/>
+      <c r="V10" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="X10" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C11" s="9"/>
       <c r="D11" s="2" t="s">
         <v>86</v>
       </c>
       <c r="R11" s="8" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="12" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C12" s="11" t="s">
+      <c r="V11" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="X11" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C12" s="9" t="s">
         <v>50</v>
       </c>
       <c r="D12" s="2" t="s">
@@ -1511,27 +1706,39 @@
       <c r="R12" s="8" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="13" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C13" s="11"/>
+      <c r="V12" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="X12" s="2" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C13" s="9"/>
       <c r="D13" s="2" t="s">
         <v>90</v>
       </c>
       <c r="R13" s="8" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="14" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C14" s="11"/>
+      <c r="V13" s="2" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C14" s="9"/>
       <c r="D14" s="2" t="s">
         <v>89</v>
       </c>
       <c r="R14" s="8" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="15" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C15" s="11" t="s">
+      <c r="V14" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C15" s="9" t="s">
         <v>45</v>
       </c>
       <c r="D15" s="2" t="s">
@@ -1540,199 +1747,232 @@
       <c r="R15" s="8" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="16" spans="1:20" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C16" s="11"/>
+      <c r="V15" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C16" s="9"/>
       <c r="D16" s="2" t="s">
         <v>70</v>
       </c>
       <c r="R16" s="8" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="17" spans="3:18" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C17" s="11"/>
+      <c r="V16" s="2" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="17" spans="3:22" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C17" s="9"/>
       <c r="D17" s="2" t="s">
         <v>67</v>
       </c>
       <c r="R17" s="8" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="18" spans="3:18" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C18" s="11"/>
+      <c r="V17" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="18" spans="3:22" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C18" s="9"/>
       <c r="D18" s="2" t="s">
         <v>68</v>
       </c>
       <c r="R18" s="8" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="19" spans="3:18" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="C19" s="11"/>
+      <c r="V18" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="19" spans="3:22" ht="15.6" x14ac:dyDescent="0.25">
+      <c r="C19" s="9"/>
       <c r="D19" s="2" t="s">
         <v>66</v>
       </c>
       <c r="R19" s="8" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="20" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C20" s="11"/>
+      <c r="V19" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C20" s="9"/>
       <c r="D20" s="2" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="21" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C21" s="11"/>
+      <c r="V20" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C21" s="9"/>
       <c r="D21" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="22" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C22" s="11"/>
+      <c r="V21" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C22" s="9"/>
       <c r="D22" s="2" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="23" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C23" s="11"/>
+      <c r="V22" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C23" s="9"/>
       <c r="D23" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="24" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C24" s="11"/>
+      <c r="V23" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="24" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C24" s="9"/>
       <c r="D24" s="2" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="25" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C25" s="11" t="s">
+      <c r="V24" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="25" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C25" s="9" t="s">
         <v>48</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="26" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C26" s="11"/>
+      <c r="V25" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="26" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C26" s="9"/>
       <c r="D26" s="2" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="27" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C27" s="11"/>
+    <row r="27" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C27" s="9"/>
       <c r="D27" s="2" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C28" s="11" t="s">
+    <row r="28" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C28" s="9" t="s">
         <v>51</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="29" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C29" s="11"/>
+    <row r="29" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C29" s="9"/>
       <c r="D29" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="30" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C30" s="11"/>
+    <row r="30" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C30" s="9"/>
       <c r="D30" s="2" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C31" s="11"/>
+    <row r="31" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C31" s="9"/>
       <c r="D31" s="2" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C32" s="11"/>
+    <row r="32" spans="3:22" x14ac:dyDescent="0.25">
+      <c r="C32" s="9"/>
       <c r="D32" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="33" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C33" s="11"/>
+      <c r="C33" s="9"/>
       <c r="D33" s="2" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="34" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C34" s="11"/>
+      <c r="C34" s="9"/>
       <c r="D34" s="2" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="35" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C35" s="11"/>
+      <c r="C35" s="9"/>
       <c r="D35" s="2" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="36" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C36" s="11"/>
+      <c r="C36" s="9"/>
       <c r="D36" s="2" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="37" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C37" s="11"/>
+      <c r="C37" s="9"/>
       <c r="D37" s="2" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="38" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C38" s="11"/>
+      <c r="C38" s="9"/>
       <c r="D38" s="2" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="39" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C39" s="11"/>
+      <c r="C39" s="9"/>
       <c r="D39" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="40" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C40" s="11"/>
+      <c r="C40" s="9"/>
       <c r="D40" s="2" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="41" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C41" s="11"/>
+      <c r="C41" s="9"/>
       <c r="D41" s="2" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="42" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C42" s="11"/>
+      <c r="C42" s="9"/>
       <c r="D42" s="2" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="43" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C43" s="11"/>
+      <c r="C43" s="9"/>
       <c r="D43" s="2" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="44" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C44" s="11"/>
+      <c r="C44" s="9"/>
       <c r="D44" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="45" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C45" s="11" t="s">
+      <c r="C45" s="9" t="s">
         <v>52</v>
       </c>
       <c r="D45" s="2" t="s">
@@ -1740,25 +1980,25 @@
       </c>
     </row>
     <row r="46" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C46" s="11"/>
+      <c r="C46" s="9"/>
       <c r="D46" s="2" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="47" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C47" s="11"/>
+      <c r="C47" s="9"/>
       <c r="D47" s="2" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="48" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C48" s="11"/>
+      <c r="C48" s="9"/>
       <c r="D48" s="2" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="49" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C49" s="11" t="s">
+      <c r="C49" s="9" t="s">
         <v>47</v>
       </c>
       <c r="D49" s="2" t="s">
@@ -1766,25 +2006,25 @@
       </c>
     </row>
     <row r="50" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C50" s="11"/>
+      <c r="C50" s="9"/>
       <c r="D50" s="2" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="51" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C51" s="11"/>
+      <c r="C51" s="9"/>
       <c r="D51" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="52" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C52" s="11"/>
+      <c r="C52" s="9"/>
       <c r="D52" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="53" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="9" t="s">
         <v>43</v>
       </c>
       <c r="D53" s="2" t="s">
@@ -1792,71 +2032,71 @@
       </c>
     </row>
     <row r="54" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C54" s="11"/>
+      <c r="C54" s="9"/>
       <c r="D54" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="55" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C55" s="11"/>
+      <c r="C55" s="9"/>
       <c r="D55" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="56" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C56" s="11"/>
+      <c r="C56" s="9"/>
       <c r="D56" s="2" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="57" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C57" s="11"/>
+      <c r="C57" s="9"/>
       <c r="D57" s="2" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="58" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C58" s="11"/>
+      <c r="C58" s="9"/>
       <c r="D58" s="2" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="59" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C59" s="11"/>
+      <c r="C59" s="9"/>
       <c r="D59" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="60" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C60" s="11"/>
+      <c r="C60" s="9"/>
       <c r="D60" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="61" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C61" s="11"/>
+      <c r="C61" s="9"/>
       <c r="D61" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="62" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C62" s="11"/>
+      <c r="C62" s="9"/>
       <c r="D62" s="2" t="s">
         <v>59</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="C15:C24"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="C28:C44"/>
+    <mergeCell ref="C45:C48"/>
     <mergeCell ref="C49:C52"/>
     <mergeCell ref="C53:C62"/>
     <mergeCell ref="C2:C8"/>
     <mergeCell ref="C9:C11"/>
     <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="C15:C24"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="C28:C44"/>
-    <mergeCell ref="C45:C48"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>